<commit_message>
Fix Yuliia Khodorovska 16 Sep shift to B
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LsGdck9uUBqMn7Bw6wMhA5
</commit_message>
<xml_diff>
--- a/Personel_Devam_Cizelgesi_Eylul_2026_YULIIA_KHODOROVSKA.xlsx
+++ b/Personel_Devam_Cizelgesi_Eylul_2026_YULIIA_KHODOROVSKA.xlsx
@@ -1528,7 +1528,7 @@
       </c>
       <c r="C30" s="28" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D30" s="6" t="n"/>
@@ -1538,7 +1538,7 @@
       <c r="H30" s="6" t="n"/>
       <c r="I30" s="28" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="J30" s="9" t="n"/>

</xml_diff>